<commit_message>
Minor fixation 12 Mar 2026
</commit_message>
<xml_diff>
--- a/AIS/wwwroot/Images/Page ID.xlsx
+++ b/AIS/wwwroot/Images/Page ID.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2182" uniqueCount="957">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2202" uniqueCount="965">
   <si>
     <t>PAGE_NAME</t>
   </si>
@@ -2868,37 +2868,61 @@
     <t>MANReport/AuditObjectiveScope</t>
   </si>
   <si>
-    <t>FFR PART 1</t>
-  </si>
-  <si>
-    <t>IID/FFR_PART1</t>
-  </si>
-  <si>
-    <t>FFR_PART1</t>
-  </si>
-  <si>
-    <t>FFR PART 2</t>
-  </si>
-  <si>
-    <t>IID/FFR_PART2</t>
-  </si>
-  <si>
-    <t>FFR_PART2</t>
-  </si>
-  <si>
-    <t>FFR PART 3</t>
-  </si>
-  <si>
-    <t>IID/FFR_PART3</t>
-  </si>
-  <si>
-    <t>FFR_PART3</t>
-  </si>
-  <si>
     <t>TaskListIID</t>
   </si>
   <si>
     <t>IID/TaskListIID</t>
+  </si>
+  <si>
+    <t>Planning Dash Board</t>
+  </si>
+  <si>
+    <t>Planning/Planning</t>
+  </si>
+  <si>
+    <t>Field Audit Dashboard</t>
+  </si>
+  <si>
+    <t>FieldAudit/AR_Dashboard</t>
+  </si>
+  <si>
+    <t>AR_Dashboard</t>
+  </si>
+  <si>
+    <t>FieldAudit/BO_Dashboard</t>
+  </si>
+  <si>
+    <t>BO_Dashboard</t>
+  </si>
+  <si>
+    <t>IID/MonitoringDashboard</t>
+  </si>
+  <si>
+    <t>IID Monitoring Dashboard</t>
+  </si>
+  <si>
+    <t>MonitoringDashboard</t>
+  </si>
+  <si>
+    <t>InquiryReportReadOnly</t>
+  </si>
+  <si>
+    <t>Inquiry Report ReadOnly</t>
+  </si>
+  <si>
+    <t>IID/InquiryReportReadOnly</t>
+  </si>
+  <si>
+    <t>FieldAuditReport/Engagements</t>
+  </si>
+  <si>
+    <t>Engagements</t>
+  </si>
+  <si>
+    <t>ObservationPdf/ObservationPrint</t>
+  </si>
+  <si>
+    <t>ObservationPrint</t>
   </si>
 </sst>
 </file>
@@ -2949,10 +2973,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3233,7 +3259,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K314"/>
+  <dimension ref="A1:K318"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="13.2" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.77734375" style="1"/>
@@ -13495,13 +13521,13 @@
         <v>7</v>
       </c>
       <c r="D311" s="1" t="s">
-        <v>946</v>
+        <v>956</v>
       </c>
       <c r="E311" s="1" t="s">
         <v>886</v>
       </c>
       <c r="F311" s="1" t="s">
-        <v>947</v>
+        <v>955</v>
       </c>
       <c r="G311" s="1">
         <v>1</v>
@@ -13513,7 +13539,7 @@
         <v>0</v>
       </c>
       <c r="K311" s="1" t="s">
-        <v>948</v>
+        <v>957</v>
       </c>
     </row>
     <row r="312" spans="1:11" x14ac:dyDescent="0.3">
@@ -13528,13 +13554,13 @@
         <v>7</v>
       </c>
       <c r="D312" s="1" t="s">
-        <v>949</v>
+        <v>959</v>
       </c>
       <c r="E312" s="1" t="s">
         <v>886</v>
       </c>
       <c r="F312" s="1" t="s">
-        <v>950</v>
+        <v>960</v>
       </c>
       <c r="G312" s="1">
         <v>2</v>
@@ -13546,28 +13572,28 @@
         <v>0</v>
       </c>
       <c r="K312" s="1" t="s">
-        <v>951</v>
+        <v>958</v>
       </c>
     </row>
     <row r="313" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A313" s="1">
         <f>B313</f>
-        <v>408</v>
+        <v>398</v>
       </c>
       <c r="B313" s="1">
-        <v>408</v>
+        <v>398</v>
       </c>
       <c r="C313" s="1">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D313" s="1" t="s">
-        <v>952</v>
+        <v>962</v>
       </c>
       <c r="E313" s="1" t="s">
-        <v>886</v>
+        <v>883</v>
       </c>
       <c r="F313" s="1" t="s">
-        <v>953</v>
+        <v>961</v>
       </c>
       <c r="G313" s="1">
         <v>3</v>
@@ -13579,7 +13605,7 @@
         <v>0</v>
       </c>
       <c r="K313" s="1" t="s">
-        <v>954</v>
+        <v>962</v>
       </c>
     </row>
     <row r="314" spans="1:11" x14ac:dyDescent="0.3">
@@ -13594,13 +13620,13 @@
         <v>7</v>
       </c>
       <c r="D314" s="1" t="s">
-        <v>955</v>
+        <v>946</v>
       </c>
       <c r="E314" s="1" t="s">
         <v>886</v>
       </c>
       <c r="F314" s="1" t="s">
-        <v>956</v>
+        <v>947</v>
       </c>
       <c r="G314" s="1">
         <v>13</v>
@@ -13612,7 +13638,142 @@
         <v>0</v>
       </c>
       <c r="K314" s="1" t="s">
-        <v>955</v>
+        <v>946</v>
+      </c>
+    </row>
+    <row r="315" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A315" s="4">
+        <f t="shared" ref="A315:A318" si="5">B315</f>
+        <v>410</v>
+      </c>
+      <c r="B315" s="4">
+        <v>410</v>
+      </c>
+      <c r="C315" s="4">
+        <v>3</v>
+      </c>
+      <c r="D315" s="4" t="s">
+        <v>948</v>
+      </c>
+      <c r="E315" s="4" t="s">
+        <v>881</v>
+      </c>
+      <c r="F315" s="4" t="s">
+        <v>949</v>
+      </c>
+      <c r="G315" s="4">
+        <v>1</v>
+      </c>
+      <c r="H315" s="4" t="s">
+        <v>770</v>
+      </c>
+      <c r="I315" s="4">
+        <v>0</v>
+      </c>
+      <c r="J315" s="3"/>
+      <c r="K315" s="4" t="s">
+        <v>888</v>
+      </c>
+    </row>
+    <row r="316" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A316" s="4">
+        <f t="shared" si="5"/>
+        <v>411</v>
+      </c>
+      <c r="B316" s="4">
+        <v>411</v>
+      </c>
+      <c r="C316" s="4">
+        <v>8</v>
+      </c>
+      <c r="D316" s="4" t="s">
+        <v>950</v>
+      </c>
+      <c r="E316" s="4" t="s">
+        <v>883</v>
+      </c>
+      <c r="F316" s="4" t="s">
+        <v>951</v>
+      </c>
+      <c r="G316" s="4">
+        <v>1</v>
+      </c>
+      <c r="H316" s="4" t="s">
+        <v>770</v>
+      </c>
+      <c r="I316" s="4">
+        <v>0</v>
+      </c>
+      <c r="J316" s="4"/>
+      <c r="K316" s="4" t="s">
+        <v>952</v>
+      </c>
+    </row>
+    <row r="317" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A317" s="4">
+        <f t="shared" si="5"/>
+        <v>412</v>
+      </c>
+      <c r="B317" s="4">
+        <v>412</v>
+      </c>
+      <c r="C317" s="4">
+        <v>8</v>
+      </c>
+      <c r="D317" s="4" t="s">
+        <v>950</v>
+      </c>
+      <c r="E317" s="4" t="s">
+        <v>883</v>
+      </c>
+      <c r="F317" s="4" t="s">
+        <v>953</v>
+      </c>
+      <c r="G317" s="4">
+        <v>1</v>
+      </c>
+      <c r="H317" s="4" t="s">
+        <v>770</v>
+      </c>
+      <c r="I317" s="4">
+        <v>0</v>
+      </c>
+      <c r="J317" s="4"/>
+      <c r="K317" s="4" t="s">
+        <v>954</v>
+      </c>
+    </row>
+    <row r="318" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A318" s="4">
+        <f t="shared" si="5"/>
+        <v>398</v>
+      </c>
+      <c r="B318" s="1">
+        <v>398</v>
+      </c>
+      <c r="C318" s="1">
+        <v>8</v>
+      </c>
+      <c r="D318" s="1" t="s">
+        <v>964</v>
+      </c>
+      <c r="E318" s="4" t="s">
+        <v>883</v>
+      </c>
+      <c r="F318" s="1" t="s">
+        <v>963</v>
+      </c>
+      <c r="G318" s="4">
+        <v>1</v>
+      </c>
+      <c r="H318" s="4" t="s">
+        <v>770</v>
+      </c>
+      <c r="I318" s="4">
+        <v>0</v>
+      </c>
+      <c r="K318" s="1" t="s">
+        <v>964</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remodellng of whole solution
</commit_message>
<xml_diff>
--- a/AIS/wwwroot/Images/Page ID.xlsx
+++ b/AIS/wwwroot/Images/Page ID.xlsx
@@ -1,33 +1,346 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asad Ali\Documents\GitHub\HTTPS-IAS-Production\AIS\wwwroot\Images\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9072"/>
-  </bookViews>
-  <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
-  </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$K$299</definedName>
-  </definedNames>
-  <calcPr calcId="162913"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
-</workbook>
+<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <Application>Microsoft Excel</Application>
+  <DocSecurity>0</DocSecurity>
+  <ScaleCrop>false</ScaleCrop>
+  <HeadingPairs>
+    <vt:vector size="2" baseType="variant">
+      <vt:variant>
+        <vt:lpstr>Worksheets</vt:lpstr>
+      </vt:variant>
+      <vt:variant>
+        <vt:i4>2</vt:i4>
+      </vt:variant>
+    </vt:vector>
+  </HeadingPairs>
+  <TitlesOfParts>
+    <vt:vector size="2" baseType="lpstr">
+      <vt:lpstr>Sheet1</vt:lpstr>
+      <vt:lpstr>Sheet2</vt:lpstr>
+    </vt:vector>
+  </TitlesOfParts>
+  <Company/>
+  <LinksUpToDate>false</LinksUpToDate>
+  <SharedDoc>false</SharedDoc>
+  <HyperlinksChanged>false</HyperlinksChanged>
+  <AppVersion>16.0300</AppVersion>
+</Properties>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <dc:creator>AAA</dc:creator>
+  <cp:lastModifiedBy>Asad Ali Chaudhry</cp:lastModifiedBy>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2025-08-09T21:54:51Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-03-27T05:54:50Z</dcterms:modified>
+</cp:coreProperties>
+</file>
+
+<file path=xl\calcChain.xml><?xml version="1.0" encoding="utf-8"?>
+<calcChain xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <c r="A322" i="1" l="1"/>
+  <c r="A321" i="1"/>
+  <c r="A320" i="1"/>
+  <c r="A319" i="1" l="1"/>
+  <c r="A315" i="1" l="1"/>
+  <c r="A316" i="1"/>
+  <c r="A317" i="1"/>
+  <c r="A318" i="1"/>
+  <c r="A314" i="1" l="1"/>
+  <c r="A313" i="1" l="1"/>
+  <c r="A312" i="1"/>
+  <c r="A311" i="1"/>
+  <c r="A142" i="1" l="1"/>
+  <c r="A150" i="1"/>
+  <c r="A143" i="1"/>
+  <c r="A157" i="1"/>
+  <c r="A148" i="1"/>
+  <c r="A149" i="1"/>
+  <c r="A156" i="1"/>
+  <c r="A158" i="1"/>
+  <c r="A61" i="1"/>
+  <c r="A60" i="1"/>
+  <c r="A62" i="1"/>
+  <c r="A66" i="1"/>
+  <c r="A65" i="1"/>
+  <c r="A58" i="1"/>
+  <c r="A175" i="1"/>
+  <c r="A233" i="1"/>
+  <c r="A227" i="1"/>
+  <c r="A188" i="1"/>
+  <c r="A231" i="1"/>
+  <c r="A225" i="1"/>
+  <c r="A171" i="1"/>
+  <c r="A267" i="1"/>
+  <c r="A275" i="1"/>
+  <c r="A280" i="1"/>
+  <c r="A274" i="1"/>
+  <c r="A273" i="1"/>
+  <c r="A144" i="1"/>
+  <c r="A145" i="1"/>
+  <c r="A22" i="1"/>
+  <c r="A21" i="1"/>
+  <c r="A14" i="1"/>
+  <c r="A5" i="1"/>
+  <c r="A4" i="1"/>
+  <c r="A28" i="1"/>
+  <c r="A153" i="1"/>
+  <c r="A31" i="1"/>
+  <c r="A17" i="1"/>
+  <c r="A30" i="1"/>
+  <c r="A29" i="1"/>
+  <c r="A50" i="1"/>
+  <c r="A13" i="1"/>
+  <c r="A12" i="1"/>
+  <c r="A18" i="1"/>
+  <c r="A19" i="1"/>
+  <c r="A64" i="1"/>
+  <c r="A155" i="1"/>
+  <c r="A241" i="1"/>
+  <c r="A57" i="1"/>
+  <c r="A245" i="1"/>
+  <c r="A154" i="1"/>
+  <c r="A240" i="1"/>
+  <c r="A146" i="1"/>
+  <c r="A244" i="1"/>
+  <c r="A147" i="1"/>
+  <c r="A53" i="1"/>
+  <c r="A56" i="1"/>
+  <c r="A59" i="1"/>
+  <c r="A55" i="1"/>
+  <c r="A54" i="1"/>
+  <c r="A75" i="1"/>
+  <c r="A106" i="1"/>
+  <c r="A76" i="1"/>
+  <c r="A99" i="1"/>
+  <c r="A96" i="1"/>
+  <c r="A100" i="1"/>
+  <c r="A212" i="1"/>
+  <c r="A217" i="1"/>
+  <c r="A84" i="1"/>
+  <c r="A78" i="1"/>
+  <c r="A211" i="1"/>
+  <c r="A93" i="1"/>
+  <c r="A87" i="1"/>
+  <c r="A73" i="1"/>
+  <c r="A83" i="1"/>
+  <c r="A34" i="1"/>
+  <c r="A35" i="1"/>
+  <c r="A32" i="1"/>
+  <c r="A179" i="1"/>
+  <c r="A219" i="1"/>
+  <c r="A192" i="1"/>
+  <c r="A181" i="1"/>
+  <c r="A230" i="1"/>
+  <c r="A239" i="1"/>
+  <c r="A223" i="1"/>
+  <c r="A221" i="1"/>
+  <c r="A173" i="1"/>
+  <c r="A190" i="1"/>
+  <c r="A191" i="1"/>
+  <c r="A182" i="1"/>
+  <c r="A218" i="1"/>
+  <c r="A194" i="1"/>
+  <c r="A180" i="1"/>
+  <c r="A235" i="1"/>
+  <c r="A238" i="1"/>
+  <c r="A126" i="1"/>
+  <c r="A97" i="1"/>
+  <c r="A105" i="1"/>
+  <c r="A88" i="1"/>
+  <c r="A42" i="1"/>
+  <c r="A74" i="1"/>
+  <c r="A213" i="1"/>
+  <c r="A178" i="1"/>
+  <c r="A214" i="1"/>
+  <c r="A81" i="1"/>
+  <c r="A82" i="1"/>
+  <c r="A79" i="1"/>
+  <c r="A89" i="1"/>
+  <c r="A90" i="1"/>
+  <c r="A209" i="1"/>
+  <c r="A186" i="1"/>
+  <c r="A187" i="1"/>
+  <c r="A94" i="1"/>
+  <c r="A85" i="1"/>
+  <c r="A95" i="1"/>
+  <c r="A67" i="1"/>
+  <c r="A68" i="1"/>
+  <c r="A183" i="1"/>
+  <c r="A128" i="1"/>
+  <c r="A129" i="1"/>
+  <c r="A104" i="1"/>
+  <c r="A177" i="1"/>
+  <c r="A71" i="1"/>
+  <c r="A237" i="1"/>
+  <c r="A206" i="1"/>
+  <c r="A201" i="1"/>
+  <c r="A195" i="1"/>
+  <c r="A196" i="1"/>
+  <c r="A172" i="1"/>
+  <c r="A200" i="1"/>
+  <c r="A198" i="1"/>
+  <c r="A197" i="1"/>
+  <c r="A199" i="1"/>
+  <c r="A101" i="1"/>
+  <c r="A122" i="1"/>
+  <c r="A108" i="1"/>
+  <c r="A203" i="1"/>
+  <c r="A208" i="1"/>
+  <c r="A207" i="1"/>
+  <c r="A109" i="1"/>
+  <c r="A204" i="1"/>
+  <c r="A205" i="1"/>
+  <c r="A25" i="1"/>
+  <c r="A63" i="1"/>
+  <c r="A70" i="1"/>
+  <c r="A107" i="1"/>
+  <c r="A72" i="1"/>
+  <c r="A202" i="1"/>
+  <c r="A110" i="1"/>
+  <c r="A39" i="1"/>
+  <c r="A49" i="1"/>
+  <c r="A44" i="1"/>
+  <c r="A45" i="1"/>
+  <c r="A37" i="1"/>
+  <c r="A272" i="1"/>
+  <c r="A270" i="1"/>
+  <c r="A224" i="1"/>
+  <c r="A20" i="1"/>
+  <c r="A6" i="1"/>
+  <c r="A269" i="1"/>
+  <c r="A276" i="1"/>
+  <c r="A281" i="1"/>
+  <c r="A24" i="1"/>
+  <c r="A10" i="1"/>
+  <c r="A9" i="1"/>
+  <c r="A11" i="1"/>
+  <c r="A164" i="1"/>
+  <c r="A166" i="1"/>
+  <c r="A165" i="1"/>
+  <c r="A43" i="1"/>
+  <c r="A216" i="1"/>
+  <c r="A23" i="1"/>
+  <c r="A242" i="1"/>
+  <c r="A103" i="1"/>
+  <c r="A234" i="1"/>
+  <c r="A226" i="1"/>
+  <c r="A184" i="1"/>
+  <c r="A77" i="1"/>
+  <c r="A220" i="1"/>
+  <c r="A285" i="1"/>
+  <c r="A286" i="1"/>
+  <c r="A282" i="1"/>
+  <c r="A284" i="1"/>
+  <c r="A283" i="1"/>
+  <c r="A33" i="1"/>
+  <c r="A36" i="1"/>
+  <c r="A40" i="1"/>
+  <c r="A46" i="1"/>
+  <c r="A47" i="1"/>
+  <c r="A262" i="1"/>
+  <c r="A277" i="1"/>
+  <c r="A263" i="1"/>
+  <c r="A41" i="1"/>
+  <c r="A167" i="1"/>
+  <c r="A232" i="1"/>
+  <c r="A15" i="1"/>
+  <c r="A174" i="1"/>
+  <c r="A98" i="1"/>
+  <c r="A38" i="1"/>
+  <c r="A168" i="1"/>
+  <c r="A8" i="1"/>
+  <c r="A215" i="1"/>
+  <c r="A189" i="1"/>
+  <c r="A26" i="1"/>
+  <c r="A80" i="1"/>
+  <c r="A86" i="1"/>
+  <c r="A3" i="1"/>
+  <c r="A287" i="1"/>
+  <c r="A210" i="1"/>
+  <c r="A176" i="1"/>
+  <c r="A268" i="1"/>
+  <c r="A271" i="1"/>
+  <c r="A246" i="1"/>
+  <c r="A278" i="1"/>
+  <c r="A264" i="1"/>
+  <c r="A279" i="1"/>
+  <c r="A265" i="1"/>
+  <c r="A185" i="1"/>
+  <c r="A266" i="1"/>
+  <c r="A16" i="1"/>
+  <c r="A229" i="1"/>
+  <c r="A169" i="1"/>
+  <c r="A170" i="1"/>
+  <c r="A193" i="1"/>
+  <c r="A161" i="1"/>
+  <c r="A160" i="1"/>
+  <c r="A159" i="1"/>
+  <c r="A151" i="1"/>
+  <c r="A152" i="1"/>
+  <c r="A91" i="1"/>
+  <c r="A92" i="1"/>
+  <c r="A69" i="1"/>
+  <c r="A48" i="1"/>
+  <c r="A102" i="1"/>
+  <c r="A255" i="1"/>
+  <c r="A247" i="1"/>
+  <c r="A252" i="1"/>
+  <c r="A250" i="1"/>
+  <c r="A249" i="1"/>
+  <c r="A258" i="1"/>
+  <c r="A236" i="1"/>
+  <c r="A228" i="1"/>
+  <c r="A257" i="1"/>
+  <c r="A256" i="1"/>
+  <c r="A261" i="1"/>
+  <c r="A222" i="1"/>
+  <c r="A248" i="1"/>
+  <c r="A251" i="1"/>
+  <c r="A254" i="1"/>
+  <c r="A116" i="1"/>
+  <c r="A259" i="1"/>
+  <c r="A117" i="1"/>
+  <c r="A2" i="1"/>
+  <c r="A123" i="1"/>
+  <c r="A27" i="1"/>
+  <c r="A7" i="1"/>
+  <c r="A115" i="1"/>
+  <c r="A133" i="1"/>
+  <c r="A132" i="1"/>
+  <c r="A134" i="1"/>
+  <c r="A135" i="1"/>
+  <c r="A136" i="1"/>
+  <c r="A137" i="1"/>
+  <c r="A138" i="1"/>
+  <c r="A139" i="1"/>
+  <c r="A140" i="1"/>
+  <c r="A141" i="1"/>
+  <c r="A162" i="1"/>
+  <c r="A163" i="1"/>
+  <c r="A51" i="1"/>
+  <c r="A52" i="1"/>
+  <c r="A114" i="1"/>
+  <c r="A111" i="1"/>
+  <c r="A119" i="1"/>
+  <c r="A120" i="1"/>
+  <c r="A121" i="1"/>
+  <c r="A124" i="1"/>
+  <c r="A118" i="1"/>
+  <c r="A125" i="1"/>
+  <c r="A113" i="1"/>
+  <c r="A112" i="1"/>
+  <c r="A130" i="1"/>
+  <c r="A131" i="1"/>
+  <c r="A127" i="1"/>
+  <c r="A260" i="1"/>
+  <c r="A253" i="1"/>
+  <c r="A243" i="1"/>
+</calcChain>
+</file>
+
+<file path=xl\sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2222" uniqueCount="977">
   <si>
     <t>PAGE_NAME</t>
@@ -2963,7 +3276,7 @@
 </sst>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -3032,7 +3345,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -3293,7 +3606,35 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr defaultThemeVersion="164011"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asad Ali\Documents\GitHub\HTTPS-IAS-Production\AIS\wwwroot\Images\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9072"/>
+  </bookViews>
+  <sheets>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+  </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$K$299</definedName>
+  </definedNames>
+  <calcPr calcId="162913"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+  </extLst>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:K322"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="13.2" x14ac:dyDescent="0.3"/>
@@ -3413,72 +3754,6 @@
         <v>710</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A4" s="1">
-        <f t="shared" si="0"/>
-        <v>45</v>
-      </c>
-      <c r="B4" s="1">
-        <v>45</v>
-      </c>
-      <c r="C4" s="1">
-        <v>6</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>290</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>874</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>291</v>
-      </c>
-      <c r="G4" s="1">
-        <v>13</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>774</v>
-      </c>
-      <c r="I4" s="1">
-        <v>1</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>645</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A5" s="1">
-        <f t="shared" si="0"/>
-        <v>44</v>
-      </c>
-      <c r="B5" s="1">
-        <v>44</v>
-      </c>
-      <c r="C5" s="1">
-        <v>6</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>288</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>874</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>289</v>
-      </c>
-      <c r="G5" s="1">
-        <v>12</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>774</v>
-      </c>
-      <c r="I5" s="1">
-        <v>1</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>644</v>
-      </c>
-    </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <f t="shared" si="0"/>
@@ -3611,39 +3886,6 @@
         <v>706</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A10" s="1">
-        <f t="shared" si="0"/>
-        <v>216</v>
-      </c>
-      <c r="B10" s="1">
-        <v>216</v>
-      </c>
-      <c r="C10" s="1">
-        <v>10</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>383</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>874</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>384</v>
-      </c>
-      <c r="G10" s="1">
-        <v>7</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>770</v>
-      </c>
-      <c r="I10" s="1">
-        <v>0</v>
-      </c>
-      <c r="K10" s="1" t="s">
-        <v>705</v>
-      </c>
-    </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <f t="shared" si="0"/>
@@ -3842,39 +4084,6 @@
         <v>711</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A17" s="1">
-        <f t="shared" si="0"/>
-        <v>50</v>
-      </c>
-      <c r="B17" s="1">
-        <v>50</v>
-      </c>
-      <c r="C17" s="1">
-        <v>8</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>326</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>874</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>327</v>
-      </c>
-      <c r="G17" s="1">
-        <v>3</v>
-      </c>
-      <c r="H17" s="1" t="s">
-        <v>774</v>
-      </c>
-      <c r="I17" s="1">
-        <v>0</v>
-      </c>
-      <c r="K17" s="1" t="s">
-        <v>663</v>
-      </c>
-    </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <f t="shared" si="0"/>
@@ -4304,39 +4513,6 @@
         <v>692</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A31" s="1">
-        <f t="shared" si="0"/>
-        <v>48</v>
-      </c>
-      <c r="B31" s="1">
-        <v>48</v>
-      </c>
-      <c r="C31" s="1">
-        <v>8</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>324</v>
-      </c>
-      <c r="E31" s="1" t="s">
-        <v>875</v>
-      </c>
-      <c r="F31" s="1" t="s">
-        <v>325</v>
-      </c>
-      <c r="G31" s="1">
-        <v>1</v>
-      </c>
-      <c r="H31" s="1" t="s">
-        <v>770</v>
-      </c>
-      <c r="I31" s="1">
-        <v>0</v>
-      </c>
-      <c r="K31" s="1" t="s">
-        <v>662</v>
-      </c>
-    </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
         <f t="shared" si="0"/>
@@ -4667,204 +4843,6 @@
         <v>728</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A42" s="1">
-        <f t="shared" si="0"/>
-        <v>125</v>
-      </c>
-      <c r="B42" s="1">
-        <v>125</v>
-      </c>
-      <c r="C42" s="1">
-        <v>16</v>
-      </c>
-      <c r="D42" s="1" t="s">
-        <v>403</v>
-      </c>
-      <c r="E42" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F42" s="1" t="s">
-        <v>404</v>
-      </c>
-      <c r="G42" s="1">
-        <v>3</v>
-      </c>
-      <c r="H42" s="1" t="s">
-        <v>770</v>
-      </c>
-      <c r="I42" s="1">
-        <v>0</v>
-      </c>
-      <c r="K42" s="1" t="s">
-        <v>715</v>
-      </c>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A43" s="1">
-        <f t="shared" si="0"/>
-        <v>223</v>
-      </c>
-      <c r="B43" s="1">
-        <v>223</v>
-      </c>
-      <c r="C43" s="1">
-        <v>16</v>
-      </c>
-      <c r="D43" s="1" t="s">
-        <v>421</v>
-      </c>
-      <c r="E43" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F43" s="1" t="s">
-        <v>422</v>
-      </c>
-      <c r="G43" s="1">
-        <v>5</v>
-      </c>
-      <c r="H43" s="1" t="s">
-        <v>770</v>
-      </c>
-      <c r="I43" s="1">
-        <v>0</v>
-      </c>
-      <c r="K43" s="1" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A44" s="1">
-        <f t="shared" si="0"/>
-        <v>200</v>
-      </c>
-      <c r="B44" s="1">
-        <v>200</v>
-      </c>
-      <c r="C44" s="1">
-        <v>16</v>
-      </c>
-      <c r="D44" s="1" t="s">
-        <v>425</v>
-      </c>
-      <c r="E44" s="1" t="s">
-        <v>506</v>
-      </c>
-      <c r="F44" s="1" t="s">
-        <v>426</v>
-      </c>
-      <c r="G44" s="1">
-        <v>2</v>
-      </c>
-      <c r="H44" s="1" t="s">
-        <v>770</v>
-      </c>
-      <c r="I44" s="1">
-        <v>0</v>
-      </c>
-      <c r="K44" s="1" t="s">
-        <v>725</v>
-      </c>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A45" s="1">
-        <f t="shared" si="0"/>
-        <v>201</v>
-      </c>
-      <c r="B45" s="1">
-        <v>201</v>
-      </c>
-      <c r="C45" s="1">
-        <v>16</v>
-      </c>
-      <c r="D45" s="1" t="s">
-        <v>427</v>
-      </c>
-      <c r="E45" s="1" t="s">
-        <v>506</v>
-      </c>
-      <c r="F45" s="1" t="s">
-        <v>428</v>
-      </c>
-      <c r="G45" s="1">
-        <v>3</v>
-      </c>
-      <c r="H45" s="1" t="s">
-        <v>770</v>
-      </c>
-      <c r="I45" s="1">
-        <v>0</v>
-      </c>
-      <c r="K45" s="1" t="s">
-        <v>726</v>
-      </c>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A46" s="1">
-        <f t="shared" si="0"/>
-        <v>243</v>
-      </c>
-      <c r="B46" s="1">
-        <v>243</v>
-      </c>
-      <c r="C46" s="1">
-        <v>16</v>
-      </c>
-      <c r="D46" s="1" t="s">
-        <v>417</v>
-      </c>
-      <c r="E46" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F46" s="1" t="s">
-        <v>418</v>
-      </c>
-      <c r="G46" s="1">
-        <v>0</v>
-      </c>
-      <c r="H46" s="1" t="s">
-        <v>770</v>
-      </c>
-      <c r="I46" s="1">
-        <v>0</v>
-      </c>
-      <c r="K46" s="1" t="s">
-        <v>721</v>
-      </c>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A47" s="1">
-        <f t="shared" si="0"/>
-        <v>244</v>
-      </c>
-      <c r="B47" s="1">
-        <v>244</v>
-      </c>
-      <c r="C47" s="1">
-        <v>16</v>
-      </c>
-      <c r="D47" s="1" t="s">
-        <v>419</v>
-      </c>
-      <c r="E47" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F47" s="1" t="s">
-        <v>420</v>
-      </c>
-      <c r="G47" s="1">
-        <v>0</v>
-      </c>
-      <c r="H47" s="1" t="s">
-        <v>770</v>
-      </c>
-      <c r="I47" s="1">
-        <v>0</v>
-      </c>
-      <c r="K47" s="1" t="s">
-        <v>722</v>
-      </c>
-    </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A48" s="1">
         <f t="shared" si="0"/>
@@ -5360,39 +5338,6 @@
         <v>527</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A63" s="1">
-        <f t="shared" si="0"/>
-        <v>192</v>
-      </c>
-      <c r="B63" s="1">
-        <v>192</v>
-      </c>
-      <c r="C63" s="1">
-        <v>4</v>
-      </c>
-      <c r="D63" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="E63" s="1" t="s">
-        <v>882</v>
-      </c>
-      <c r="F63" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="G63" s="1">
-        <v>2</v>
-      </c>
-      <c r="H63" s="1" t="s">
-        <v>770</v>
-      </c>
-      <c r="I63" s="1">
-        <v>0</v>
-      </c>
-      <c r="K63" s="1" t="s">
-        <v>559</v>
-      </c>
-    </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A64" s="1">
         <f t="shared" si="0"/>
@@ -5426,39 +5371,6 @@
         <v>784</v>
       </c>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A65" s="1">
-        <f t="shared" ref="A65:A118" si="1">B65</f>
-        <v>18</v>
-      </c>
-      <c r="B65" s="1">
-        <v>18</v>
-      </c>
-      <c r="C65" s="1">
-        <v>4</v>
-      </c>
-      <c r="D65" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="E65" s="1" t="s">
-        <v>882</v>
-      </c>
-      <c r="F65" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="G65" s="1">
-        <v>4</v>
-      </c>
-      <c r="H65" s="1" t="s">
-        <v>770</v>
-      </c>
-      <c r="I65" s="1">
-        <v>1</v>
-      </c>
-      <c r="K65" s="1" t="s">
-        <v>529</v>
-      </c>
-    </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A66" s="1">
         <f t="shared" si="1"/>
@@ -5591,138 +5503,6 @@
         <v>568</v>
       </c>
     </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A70" s="1">
-        <f t="shared" si="1"/>
-        <v>193</v>
-      </c>
-      <c r="B70" s="1">
-        <v>193</v>
-      </c>
-      <c r="C70" s="1">
-        <v>4</v>
-      </c>
-      <c r="D70" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="E70" s="1" t="s">
-        <v>882</v>
-      </c>
-      <c r="F70" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="G70" s="1">
-        <v>3</v>
-      </c>
-      <c r="H70" s="1" t="s">
-        <v>770</v>
-      </c>
-      <c r="I70" s="1">
-        <v>0</v>
-      </c>
-      <c r="K70" s="1" t="s">
-        <v>560</v>
-      </c>
-    </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A71" s="1">
-        <f t="shared" si="1"/>
-        <v>169</v>
-      </c>
-      <c r="B71" s="1">
-        <v>169</v>
-      </c>
-      <c r="C71" s="1">
-        <v>19</v>
-      </c>
-      <c r="D71" s="1" t="s">
-        <v>438</v>
-      </c>
-      <c r="E71" s="1" t="s">
-        <v>882</v>
-      </c>
-      <c r="F71" s="1" t="s">
-        <v>439</v>
-      </c>
-      <c r="G71" s="1">
-        <v>8</v>
-      </c>
-      <c r="H71" s="1" t="s">
-        <v>770</v>
-      </c>
-      <c r="I71" s="1">
-        <v>0</v>
-      </c>
-      <c r="K71" s="1" t="s">
-        <v>731</v>
-      </c>
-    </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A72" s="1">
-        <f t="shared" si="1"/>
-        <v>195</v>
-      </c>
-      <c r="B72" s="1">
-        <v>195</v>
-      </c>
-      <c r="C72" s="1">
-        <v>4</v>
-      </c>
-      <c r="D72" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="E72" s="1" t="s">
-        <v>882</v>
-      </c>
-      <c r="F72" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="G72" s="1">
-        <v>5</v>
-      </c>
-      <c r="H72" s="1" t="s">
-        <v>770</v>
-      </c>
-      <c r="I72" s="1">
-        <v>0</v>
-      </c>
-      <c r="K72" s="1" t="s">
-        <v>562</v>
-      </c>
-    </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A73" s="1">
-        <f t="shared" si="1"/>
-        <v>88</v>
-      </c>
-      <c r="B73" s="1">
-        <v>88</v>
-      </c>
-      <c r="C73" s="1">
-        <v>4</v>
-      </c>
-      <c r="D73" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="E73" s="1" t="s">
-        <v>882</v>
-      </c>
-      <c r="F73" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="G73" s="1">
-        <v>21</v>
-      </c>
-      <c r="H73" s="1" t="s">
-        <v>770</v>
-      </c>
-      <c r="I73" s="1">
-        <v>1</v>
-      </c>
-      <c r="K73" s="1" t="s">
-        <v>539</v>
-      </c>
-    </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A74" s="1">
         <f t="shared" si="1"/>
@@ -5954,105 +5734,6 @@
         <v>570</v>
       </c>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A81" s="1">
-        <f t="shared" si="1"/>
-        <v>148</v>
-      </c>
-      <c r="B81" s="1">
-        <v>148</v>
-      </c>
-      <c r="C81" s="1">
-        <v>4</v>
-      </c>
-      <c r="D81" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="E81" s="1" t="s">
-        <v>882</v>
-      </c>
-      <c r="F81" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="G81" s="1">
-        <v>5</v>
-      </c>
-      <c r="H81" s="1" t="s">
-        <v>774</v>
-      </c>
-      <c r="I81" s="1">
-        <v>1</v>
-      </c>
-      <c r="K81" s="1" t="s">
-        <v>547</v>
-      </c>
-    </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A82" s="1">
-        <f t="shared" si="1"/>
-        <v>149</v>
-      </c>
-      <c r="B82" s="1">
-        <v>149</v>
-      </c>
-      <c r="C82" s="1">
-        <v>4</v>
-      </c>
-      <c r="D82" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="E82" s="1" t="s">
-        <v>882</v>
-      </c>
-      <c r="F82" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="G82" s="1">
-        <v>6</v>
-      </c>
-      <c r="H82" s="1" t="s">
-        <v>770</v>
-      </c>
-      <c r="I82" s="1">
-        <v>1</v>
-      </c>
-      <c r="K82" s="1" t="s">
-        <v>548</v>
-      </c>
-    </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A83" s="1">
-        <f t="shared" si="1"/>
-        <v>89</v>
-      </c>
-      <c r="B83" s="1">
-        <v>89</v>
-      </c>
-      <c r="C83" s="1">
-        <v>4</v>
-      </c>
-      <c r="D83" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="E83" s="1" t="s">
-        <v>882</v>
-      </c>
-      <c r="F83" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="G83" s="1">
-        <v>22</v>
-      </c>
-      <c r="H83" s="1" t="s">
-        <v>770</v>
-      </c>
-      <c r="I83" s="1">
-        <v>1</v>
-      </c>
-      <c r="K83" s="1" t="s">
-        <v>541</v>
-      </c>
-    </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A84" s="1">
         <f t="shared" si="1"/>
@@ -6152,138 +5833,6 @@
         <v>571</v>
       </c>
     </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A87" s="1">
-        <f t="shared" si="1"/>
-        <v>87</v>
-      </c>
-      <c r="B87" s="1">
-        <v>87</v>
-      </c>
-      <c r="C87" s="1">
-        <v>4</v>
-      </c>
-      <c r="D87" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="E87" s="1" t="s">
-        <v>882</v>
-      </c>
-      <c r="F87" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="G87" s="1">
-        <v>20</v>
-      </c>
-      <c r="H87" s="1" t="s">
-        <v>770</v>
-      </c>
-      <c r="I87" s="1">
-        <v>1</v>
-      </c>
-      <c r="K87" s="1" t="s">
-        <v>538</v>
-      </c>
-    </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A88" s="1">
-        <f t="shared" si="1"/>
-        <v>124</v>
-      </c>
-      <c r="B88" s="1">
-        <v>124</v>
-      </c>
-      <c r="C88" s="1">
-        <v>4</v>
-      </c>
-      <c r="D88" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="E88" s="1" t="s">
-        <v>882</v>
-      </c>
-      <c r="F88" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="G88" s="1">
-        <v>6</v>
-      </c>
-      <c r="H88" s="1" t="s">
-        <v>770</v>
-      </c>
-      <c r="I88" s="1">
-        <v>1</v>
-      </c>
-      <c r="K88" s="1" t="s">
-        <v>535</v>
-      </c>
-    </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A89" s="1">
-        <f t="shared" si="1"/>
-        <v>151</v>
-      </c>
-      <c r="B89" s="1">
-        <v>151</v>
-      </c>
-      <c r="C89" s="1">
-        <v>4</v>
-      </c>
-      <c r="D89" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="E89" s="1" t="s">
-        <v>882</v>
-      </c>
-      <c r="F89" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="G89" s="1">
-        <v>20</v>
-      </c>
-      <c r="H89" s="1" t="s">
-        <v>770</v>
-      </c>
-      <c r="I89" s="1">
-        <v>1</v>
-      </c>
-      <c r="K89" s="1" t="s">
-        <v>550</v>
-      </c>
-    </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A90" s="1">
-        <f t="shared" si="1"/>
-        <v>152</v>
-      </c>
-      <c r="B90" s="1">
-        <v>152</v>
-      </c>
-      <c r="C90" s="1">
-        <v>4</v>
-      </c>
-      <c r="D90" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="E90" s="1" t="s">
-        <v>882</v>
-      </c>
-      <c r="F90" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="G90" s="1">
-        <v>21</v>
-      </c>
-      <c r="H90" s="1" t="s">
-        <v>770</v>
-      </c>
-      <c r="I90" s="1">
-        <v>1</v>
-      </c>
-      <c r="K90" s="1" t="s">
-        <v>551</v>
-      </c>
-    </row>
     <row r="91" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A91" s="1">
         <f t="shared" si="1"/>
@@ -6515,105 +6064,6 @@
         <v>542</v>
       </c>
     </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A98" s="1">
-        <f t="shared" si="1"/>
-        <v>253</v>
-      </c>
-      <c r="B98" s="1">
-        <v>253</v>
-      </c>
-      <c r="C98" s="1">
-        <v>4</v>
-      </c>
-      <c r="D98" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="E98" s="1" t="s">
-        <v>882</v>
-      </c>
-      <c r="F98" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="G98" s="1">
-        <v>1</v>
-      </c>
-      <c r="H98" s="1" t="s">
-        <v>770</v>
-      </c>
-      <c r="I98" s="1">
-        <v>1</v>
-      </c>
-      <c r="K98" s="1" t="s">
-        <v>557</v>
-      </c>
-    </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A99" s="1">
-        <f t="shared" si="1"/>
-        <v>78</v>
-      </c>
-      <c r="B99" s="1">
-        <v>78</v>
-      </c>
-      <c r="C99" s="1">
-        <v>4</v>
-      </c>
-      <c r="D99" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="E99" s="1" t="s">
-        <v>882</v>
-      </c>
-      <c r="F99" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="G99" s="1">
-        <v>3</v>
-      </c>
-      <c r="H99" s="1" t="s">
-        <v>770</v>
-      </c>
-      <c r="I99" s="1">
-        <v>0</v>
-      </c>
-      <c r="K99" s="1" t="s">
-        <v>525</v>
-      </c>
-    </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A100" s="1">
-        <f t="shared" si="1"/>
-        <v>80</v>
-      </c>
-      <c r="B100" s="1">
-        <v>80</v>
-      </c>
-      <c r="C100" s="1">
-        <v>4</v>
-      </c>
-      <c r="D100" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="E100" s="1" t="s">
-        <v>882</v>
-      </c>
-      <c r="F100" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="G100" s="1">
-        <v>9</v>
-      </c>
-      <c r="H100" s="1" t="s">
-        <v>770</v>
-      </c>
-      <c r="I100" s="1">
-        <v>0</v>
-      </c>
-      <c r="K100" s="1" t="s">
-        <v>536</v>
-      </c>
-    </row>
     <row r="101" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A101" s="1">
         <f t="shared" si="1"/>
@@ -6713,72 +6163,6 @@
         <v>564</v>
       </c>
     </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A104" s="1">
-        <f t="shared" si="1"/>
-        <v>167</v>
-      </c>
-      <c r="B104" s="1">
-        <v>167</v>
-      </c>
-      <c r="C104" s="1">
-        <v>19</v>
-      </c>
-      <c r="D104" s="1" t="s">
-        <v>440</v>
-      </c>
-      <c r="E104" s="1" t="s">
-        <v>882</v>
-      </c>
-      <c r="F104" s="1" t="s">
-        <v>441</v>
-      </c>
-      <c r="G104" s="1">
-        <v>7</v>
-      </c>
-      <c r="H104" s="1" t="s">
-        <v>770</v>
-      </c>
-      <c r="I104" s="1">
-        <v>0</v>
-      </c>
-      <c r="K104" s="1" t="s">
-        <v>732</v>
-      </c>
-    </row>
-    <row r="105" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A105" s="1">
-        <f t="shared" si="1"/>
-        <v>123</v>
-      </c>
-      <c r="B105" s="1">
-        <v>123</v>
-      </c>
-      <c r="C105" s="1">
-        <v>4</v>
-      </c>
-      <c r="D105" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E105" s="1" t="s">
-        <v>882</v>
-      </c>
-      <c r="F105" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="G105" s="1">
-        <v>6</v>
-      </c>
-      <c r="H105" s="1" t="s">
-        <v>770</v>
-      </c>
-      <c r="I105" s="1">
-        <v>1</v>
-      </c>
-      <c r="K105" s="1" t="s">
-        <v>543</v>
-      </c>
-    </row>
     <row r="106" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A106" s="1">
         <f t="shared" si="1"/>
@@ -6812,138 +6196,6 @@
         <v>523</v>
       </c>
     </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A107" s="1">
-        <f t="shared" si="1"/>
-        <v>194</v>
-      </c>
-      <c r="B107" s="1">
-        <v>194</v>
-      </c>
-      <c r="C107" s="1">
-        <v>4</v>
-      </c>
-      <c r="D107" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="E107" s="1" t="s">
-        <v>882</v>
-      </c>
-      <c r="F107" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="G107" s="1">
-        <v>4</v>
-      </c>
-      <c r="H107" s="1" t="s">
-        <v>770</v>
-      </c>
-      <c r="I107" s="1">
-        <v>0</v>
-      </c>
-      <c r="K107" s="1" t="s">
-        <v>561</v>
-      </c>
-    </row>
-    <row r="108" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A108" s="1">
-        <f t="shared" si="1"/>
-        <v>183</v>
-      </c>
-      <c r="B108" s="1">
-        <v>183</v>
-      </c>
-      <c r="C108" s="1">
-        <v>4</v>
-      </c>
-      <c r="D108" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="E108" s="1" t="s">
-        <v>882</v>
-      </c>
-      <c r="F108" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="G108" s="1">
-        <v>19</v>
-      </c>
-      <c r="H108" s="1" t="s">
-        <v>770</v>
-      </c>
-      <c r="I108" s="1">
-        <v>0</v>
-      </c>
-      <c r="K108" s="1" t="s">
-        <v>556</v>
-      </c>
-    </row>
-    <row r="109" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A109" s="1">
-        <f t="shared" si="1"/>
-        <v>188</v>
-      </c>
-      <c r="B109" s="1">
-        <v>188</v>
-      </c>
-      <c r="C109" s="1">
-        <v>4</v>
-      </c>
-      <c r="D109" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="E109" s="1" t="s">
-        <v>882</v>
-      </c>
-      <c r="F109" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="G109" s="1">
-        <v>20</v>
-      </c>
-      <c r="H109" s="1" t="s">
-        <v>770</v>
-      </c>
-      <c r="I109" s="1">
-        <v>0</v>
-      </c>
-      <c r="K109" s="1" t="s">
-        <v>558</v>
-      </c>
-    </row>
-    <row r="110" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A110" s="1">
-        <f t="shared" si="1"/>
-        <v>197</v>
-      </c>
-      <c r="B110" s="1">
-        <v>197</v>
-      </c>
-      <c r="C110" s="1">
-        <v>4</v>
-      </c>
-      <c r="D110" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="E110" s="1" t="s">
-        <v>882</v>
-      </c>
-      <c r="F110" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="G110" s="1">
-        <v>2</v>
-      </c>
-      <c r="H110" s="1" t="s">
-        <v>770</v>
-      </c>
-      <c r="I110" s="1">
-        <v>0</v>
-      </c>
-      <c r="K110" s="1" t="s">
-        <v>563</v>
-      </c>
-    </row>
     <row r="111" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A111" s="1">
         <f t="shared" si="1"/>
@@ -7310,39 +6562,6 @@
         <v>667</v>
       </c>
     </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A122" s="1">
-        <f t="shared" si="2"/>
-        <v>182</v>
-      </c>
-      <c r="B122" s="1">
-        <v>182</v>
-      </c>
-      <c r="C122" s="1">
-        <v>18</v>
-      </c>
-      <c r="D122" s="1" t="s">
-        <v>435</v>
-      </c>
-      <c r="E122" s="1" t="s">
-        <v>883</v>
-      </c>
-      <c r="F122" s="1" t="s">
-        <v>436</v>
-      </c>
-      <c r="G122" s="1">
-        <v>1</v>
-      </c>
-      <c r="H122" s="1" t="s">
-        <v>770</v>
-      </c>
-      <c r="I122" s="1">
-        <v>0</v>
-      </c>
-      <c r="K122" s="1" t="s">
-        <v>730</v>
-      </c>
-    </row>
     <row r="123" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A123" s="1">
         <f t="shared" si="2"/>
@@ -7442,39 +6661,6 @@
         <v>664</v>
       </c>
     </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A126" s="1">
-        <f t="shared" si="2"/>
-        <v>120</v>
-      </c>
-      <c r="B126" s="1">
-        <v>120</v>
-      </c>
-      <c r="C126" s="1">
-        <v>1</v>
-      </c>
-      <c r="D126" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E126" s="1" t="s">
-        <v>885</v>
-      </c>
-      <c r="F126" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G126" s="1">
-        <v>1</v>
-      </c>
-      <c r="H126" s="1" t="s">
-        <v>770</v>
-      </c>
-      <c r="I126" s="1">
-        <v>0</v>
-      </c>
-      <c r="K126" s="1" t="s">
-        <v>506</v>
-      </c>
-    </row>
     <row r="127" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A127" s="1">
         <f t="shared" si="2"/>
@@ -8630,138 +7816,6 @@
         <v>738</v>
       </c>
     </row>
-    <row r="162" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A162" s="1">
-        <f t="shared" si="2"/>
-        <v>352</v>
-      </c>
-      <c r="B162" s="1">
-        <v>352</v>
-      </c>
-      <c r="C162" s="1">
-        <v>19</v>
-      </c>
-      <c r="D162" s="1" t="s">
-        <v>463</v>
-      </c>
-      <c r="E162" s="1" t="s">
-        <v>889</v>
-      </c>
-      <c r="F162" s="1" t="s">
-        <v>464</v>
-      </c>
-      <c r="G162" s="1">
-        <v>9</v>
-      </c>
-      <c r="H162" s="1" t="s">
-        <v>770</v>
-      </c>
-      <c r="I162" s="1">
-        <v>0</v>
-      </c>
-      <c r="K162" s="1" t="s">
-        <v>744</v>
-      </c>
-    </row>
-    <row r="163" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A163" s="1">
-        <f t="shared" si="2"/>
-        <v>353</v>
-      </c>
-      <c r="B163" s="1">
-        <v>353</v>
-      </c>
-      <c r="C163" s="1">
-        <v>19</v>
-      </c>
-      <c r="D163" s="1" t="s">
-        <v>461</v>
-      </c>
-      <c r="E163" s="1" t="s">
-        <v>889</v>
-      </c>
-      <c r="F163" s="1" t="s">
-        <v>462</v>
-      </c>
-      <c r="G163" s="1">
-        <v>10</v>
-      </c>
-      <c r="H163" s="1" t="s">
-        <v>770</v>
-      </c>
-      <c r="I163" s="1">
-        <v>0</v>
-      </c>
-      <c r="K163" s="1" t="s">
-        <v>743</v>
-      </c>
-    </row>
-    <row r="164" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A164" s="1">
-        <f t="shared" si="2"/>
-        <v>220</v>
-      </c>
-      <c r="B164" s="1">
-        <v>220</v>
-      </c>
-      <c r="C164" s="1">
-        <v>19</v>
-      </c>
-      <c r="D164" s="1" t="s">
-        <v>442</v>
-      </c>
-      <c r="E164" s="1" t="s">
-        <v>889</v>
-      </c>
-      <c r="F164" s="1" t="s">
-        <v>443</v>
-      </c>
-      <c r="G164" s="1">
-        <v>8</v>
-      </c>
-      <c r="H164" s="1" t="s">
-        <v>770</v>
-      </c>
-      <c r="I164" s="1">
-        <v>0</v>
-      </c>
-      <c r="K164" s="1" t="s">
-        <v>733</v>
-      </c>
-    </row>
-    <row r="165" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A165" s="1">
-        <f t="shared" si="2"/>
-        <v>222</v>
-      </c>
-      <c r="B165" s="1">
-        <v>222</v>
-      </c>
-      <c r="C165" s="1">
-        <v>19</v>
-      </c>
-      <c r="D165" s="1" t="s">
-        <v>446</v>
-      </c>
-      <c r="E165" s="1" t="s">
-        <v>889</v>
-      </c>
-      <c r="F165" s="1" t="s">
-        <v>447</v>
-      </c>
-      <c r="G165" s="1">
-        <v>6</v>
-      </c>
-      <c r="H165" s="1" t="s">
-        <v>770</v>
-      </c>
-      <c r="I165" s="1">
-        <v>0</v>
-      </c>
-      <c r="K165" s="1" t="s">
-        <v>735</v>
-      </c>
-    </row>
     <row r="166" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A166" s="1">
         <f t="shared" si="2"/>
@@ -10304,39 +9358,6 @@
         <v>534</v>
       </c>
     </row>
-    <row r="212" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A212" s="1">
-        <f t="shared" si="3"/>
-        <v>81</v>
-      </c>
-      <c r="B212" s="1">
-        <v>81</v>
-      </c>
-      <c r="C212" s="1">
-        <v>4</v>
-      </c>
-      <c r="D212" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="E212" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="F212" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="G212" s="1">
-        <v>15</v>
-      </c>
-      <c r="H212" s="1" t="s">
-        <v>770</v>
-      </c>
-      <c r="I212" s="1">
-        <v>1</v>
-      </c>
-      <c r="K212" s="1" t="s">
-        <v>537</v>
-      </c>
-    </row>
     <row r="213" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A213" s="1">
         <f t="shared" si="3"/>
@@ -10469,39 +9490,6 @@
         <v>618</v>
       </c>
     </row>
-    <row r="217" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A217" s="1">
-        <f t="shared" si="3"/>
-        <v>82</v>
-      </c>
-      <c r="B217" s="1">
-        <v>82</v>
-      </c>
-      <c r="C217" s="1">
-        <v>4</v>
-      </c>
-      <c r="D217" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="E217" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="F217" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="G217" s="1">
-        <v>23</v>
-      </c>
-      <c r="H217" s="1" t="s">
-        <v>770</v>
-      </c>
-      <c r="I217" s="1">
-        <v>1</v>
-      </c>
-      <c r="K217" s="1" t="s">
-        <v>531</v>
-      </c>
-    </row>
     <row r="218" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A218" s="1">
         <f t="shared" si="3"/>
@@ -12117,39 +11105,6 @@
       </c>
       <c r="K266" s="1" t="s">
         <v>658</v>
-      </c>
-    </row>
-    <row r="267" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A267" s="1">
-        <f t="shared" si="4"/>
-        <v>27</v>
-      </c>
-      <c r="B267" s="1">
-        <v>27</v>
-      </c>
-      <c r="C267" s="1">
-        <v>6</v>
-      </c>
-      <c r="D267" s="1" t="s">
-        <v>276</v>
-      </c>
-      <c r="E267" s="1" t="s">
-        <v>892</v>
-      </c>
-      <c r="F267" s="1" t="s">
-        <v>277</v>
-      </c>
-      <c r="G267" s="1">
-        <v>1</v>
-      </c>
-      <c r="H267" s="1" t="s">
-        <v>770</v>
-      </c>
-      <c r="I267" s="1">
-        <v>0</v>
-      </c>
-      <c r="K267" s="1" t="s">
-        <v>638</v>
       </c>
     </row>
     <row r="268" spans="1:11" x14ac:dyDescent="0.3">
@@ -13952,7 +12907,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C303"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>